<commit_message>
Refine Siemens trigger and valuation inputs
</commit_message>
<xml_diff>
--- a/trading/research/siegy-normalized-earnings-2026-08-07.xlsx
+++ b/trading/research/siegy-normalized-earnings-2026-08-07.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bear'!$A$1:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Base'!$A$1:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Bull'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sources'!$A$1:$C$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sources'!$A$1:$C$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Limitations'!$A$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -515,7 +515,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>$93.96 / $153.12 / $226.20</t>
+          <t>$93.43 / $152.26 / $224.93</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>12.69</v>
+        <v>12.76</v>
       </c>
     </row>
   </sheetData>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>1.16</v>
+        <v>1.1535</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -818,7 +818,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.16</v>
+        <v>1.1535</v>
       </c>
       <c r="F2" s="2">
         <f>C2/D2*E2</f>
@@ -838,7 +838,7 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>93.95999999999999</v>
+        <v>93.43000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -911,7 +911,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.16</v>
+        <v>1.1535</v>
       </c>
       <c r="F2" s="2">
         <f>C2/D2*E2</f>
@@ -931,7 +931,7 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>153.12</v>
+        <v>152.26</v>
       </c>
     </row>
   </sheetData>
@@ -1004,7 +1004,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.16</v>
+        <v>1.1535</v>
       </c>
       <c r="F2" s="2">
         <f>C2/D2*E2</f>
@@ -1024,7 +1024,7 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>226.2</v>
+        <v>224.93</v>
       </c>
     </row>
   </sheetData>
@@ -1039,10 +1039,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="72" customWidth="1" min="2" max="2"/>
     <col width="67" customWidth="1" min="3" max="3"/>
   </cols>
@@ -1115,12 +1115,48 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers spin-off timeline</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>https://press.siemens.com/global/en/pressrelease/siemens-clarifies-timeline-spin-siemens-healthineers-shares</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Targeted February 2027 shareholder vote</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Frankfurter EUR/USD reference</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://api.frankfurter.app/latest?from=EUR&amp;to=USD</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>August 7 valuation-date FX translation reference</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C4"/>
+  <autoFilter ref="A1:C6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refine Siemens trigger and valuation inputs (#324)
</commit_message>
<xml_diff>
--- a/trading/research/siegy-normalized-earnings-2026-08-07.xlsx
+++ b/trading/research/siegy-normalized-earnings-2026-08-07.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bear'!$A$1:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Base'!$A$1:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Bull'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sources'!$A$1:$C$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sources'!$A$1:$C$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Limitations'!$A$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -515,7 +515,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>$93.96 / $153.12 / $226.20</t>
+          <t>$93.43 / $152.26 / $224.93</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>12.69</v>
+        <v>12.76</v>
       </c>
     </row>
   </sheetData>
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>1.16</v>
+        <v>1.1535</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -818,7 +818,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.16</v>
+        <v>1.1535</v>
       </c>
       <c r="F2" s="2">
         <f>C2/D2*E2</f>
@@ -838,7 +838,7 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>93.95999999999999</v>
+        <v>93.43000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -911,7 +911,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.16</v>
+        <v>1.1535</v>
       </c>
       <c r="F2" s="2">
         <f>C2/D2*E2</f>
@@ -931,7 +931,7 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>153.12</v>
+        <v>152.26</v>
       </c>
     </row>
   </sheetData>
@@ -1004,7 +1004,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.16</v>
+        <v>1.1535</v>
       </c>
       <c r="F2" s="2">
         <f>C2/D2*E2</f>
@@ -1024,7 +1024,7 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>226.2</v>
+        <v>224.93</v>
       </c>
     </row>
   </sheetData>
@@ -1039,10 +1039,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="72" customWidth="1" min="2" max="2"/>
     <col width="67" customWidth="1" min="3" max="3"/>
   </cols>
@@ -1115,12 +1115,48 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers spin-off timeline</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>https://press.siemens.com/global/en/pressrelease/siemens-clarifies-timeline-spin-siemens-healthineers-shares</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Targeted February 2027 shareholder vote</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Frankfurter EUR/USD reference</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://api.frankfurter.app/latest?from=EUR&amp;to=USD</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>August 7 valuation-date FX translation reference</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C4"/>
+  <autoFilter ref="A1:C6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>